<commit_message>
Atualização de datas funcionando
</commit_message>
<xml_diff>
--- a/src/data_update/update_cards.xlsx
+++ b/src/data_update/update_cards.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="6" max="6"/>
@@ -474,44 +474,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MANTA-29977</t>
+          <t>TENSYLON-675</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Manta</t>
+          <t>Tensylon</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-29977</t>
+          <t>https://carboncars.atlassian.net/browse/TENSYLON-675</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>30442</t>
+          <t>30282</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Liberado Engenharia</t>
+          <t>A Produzir</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>⚪️REC. Encaminhado</t>
+          <t>🟢REC. Liberado</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>GWM - TANK 300 SUV - 2026</t>
+          <t>MERCEDES-BENZ - EQS 450+ SUV - 2024</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MANTA-29549</t>
+          <t>MANTA-29977</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -521,12 +521,12 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-29549</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-29977</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>30059</t>
+          <t>30442</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -541,42 +541,79 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>BMW - X1 SUV - 2026</t>
+          <t>GWM - TANK 300 SUV - 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>MANTA-29549</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Manta</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>https://carboncars.atlassian.net/browse/MANTA-29549</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>30059</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Liberado Engenharia</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>⚪️REC. Encaminhado</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>BMW - X1 SUV - 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>MANTA-28595</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Manta</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>https://carboncars.atlassian.net/browse/MANTA-28595</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>29222</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Liberado Engenharia</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>⚪️REC. Encaminhado</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>TOYOTA - COROLLA SEDAN - 2025</t>
         </is>
@@ -587,6 +624,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>